<commit_message>
Add Traditional Chinese interview materials for Deloitte demo
# Conflicts:
#	README.md
</commit_message>
<xml_diff>
--- a/industry_intelligence_agent/data/reports/industry_intelligence_demo.xlsx
+++ b/industry_intelligence_agent/data/reports/industry_intelligence_demo.xlsx
@@ -18,7 +18,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'News_Articles'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'KRI_Evidence'!$A$1:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Summary_By_Company'!$A$1:$H$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dashboard_View'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dashboard_View'!$A$3:$J$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -27,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -39,8 +39,12 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -51,6 +55,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+        <bgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -66,9 +76,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2396,7 +2407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2411,100 +2422,110 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>說明：此 Excel 由 Python 自動產生，展示顧問與 business users 可用的 KRI 風險證據、新聞訊號與 dashboard-ready 分析結果；本 MVP 使用 sample/public-style data，最終判斷需人工審閱。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B3" s="1" t="inlineStr">
         <is>
           <t>industry</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>total_news_count</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>total_kri_count</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>high_severity_kri_count</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>medium_severity_kri_count</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>low_severity_kri_count</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>overall_risk_level</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>recommended_follow_up</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>excel_follow_up_flag</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Taiwan Semiconductor Manufacturing Company</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Taiwan Semiconductor Manufacturing Company</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Taiwan semiconductor / AI server</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C4" t="n">
         <v>6</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D4" t="n">
         <v>28</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F4" t="n">
         <v>11</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G4" t="n">
         <v>16</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Validate high/medium KRI evidence with management interviews and source documents.</t>
         </is>
       </c>
-      <c r="J2">
-        <f>IF(E2&gt;0,"Priority follow-up","Monitor")</f>
+      <c r="J4">
+        <f>IF(E4&gt;0,"Priority follow-up","Monitor")</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I2"/>
+  <autoFilter ref="A3:J4"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
   <conditionalFormatting sqref="E2">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"high"</formula>
@@ -2585,6 +2606,17 @@
       <formula>"Low"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="H4">
+    <cfRule type="cellIs" priority="25" operator="equal" dxfId="0">
+      <formula>"High"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="26" operator="equal" dxfId="1">
+      <formula>"Medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="27" operator="equal" dxfId="2">
+      <formula>"Low"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>